<commit_message>
Deploy from own repo, track server SQL update scripts, add lookup templates
- deploy_hpb_server.sh: clone roxmer/HPB-AI (HPB_REPO/HPB_BRANCH/GITHUB_TOKEN
  options) into a temp folder first; PROGRAMMERS_REPO no longer used.
- Move the synthetic test patient SQL into "Populate DB/" and track the
  update_*.sql scripts that are run on the server DB (clinician role,
  lab lookup revision). .gitignore updated; scratch SQL, .bak and old
  server copies stay ignored.
- HPB_Templates: updated lookup exports; new Assessment Purpose Type,
  Freezer, LabDrawRole and Panel Context Type exports; corrected
  Resection margins file.
- Add Security_Authority_Audit_2026-10-07.md and the bulk import /
  new lookup endpoint test scripts.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/HPB_Templates/Technique_TestName_TestResult_TestUnit_export.xlsx
+++ b/HPB_Templates/Technique_TestName_TestResult_TestUnit_export.xlsx
@@ -3735,7 +3735,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Decreased</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -3795,7 +3795,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Decreased</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -7222,7 +7222,11 @@
           <t>U/mL</t>
         </is>
       </c>
-      <c r="C2" s="5" t="n"/>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
           <t>37</t>

</xml_diff>